<commit_message>
clean commit without cache files
</commit_message>
<xml_diff>
--- a/Code/Data_preprocessing/generated_data/surge_data_manual_check.xlsx
+++ b/Code/Data_preprocessing/generated_data/surge_data_manual_check.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29721"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1016" documentId="11_169D90BFD30052E6A44A05D04B5ED87656CEEB54" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D213BA7-56E3-40F5-9999-21B2E8A582B2}"/>
+  <xr:revisionPtr revIDLastSave="1070" documentId="11_169D90BFD30052E6A44A05D04B5ED87656CEEB54" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43639469-5D4E-48C3-AC28-FF83EB248340}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1628" uniqueCount="953">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1645" uniqueCount="955">
   <si>
     <t>Unique_ID</t>
   </si>
@@ -1005,6 +1005,9 @@
     <t>Florence</t>
   </si>
   <si>
+    <t>Above Normal</t>
+  </si>
+  <si>
     <t>Sep 23-28</t>
   </si>
   <si>
@@ -1080,7 +1083,7 @@
     <t>ID_86</t>
   </si>
   <si>
-    <t>tide gauge: https://tidesandcurrents.noaa.gov/stationhome.html?id=8518750</t>
+    <t>tide gauge: https://tidesandcurrents.noaa.gov/waterlevels.html?id=8518750&amp;units=standard&amp;bdate=19550816&amp;edate=19550823&amp;timezone=GMT&amp;datum=MSL&amp;interval=h&amp;action=</t>
   </si>
   <si>
     <t>ID_87</t>
@@ -1170,55 +1173,58 @@
     <t>Not Named 1959</t>
   </si>
   <si>
+    <t>gauge data from st. Petersburg: https://tidesandcurrents.noaa.gov/waterlevels.html?id=8726520&amp;units=standard&amp;bdate=19590615&amp;edate=19590622&amp;timezone=GMT&amp;datum=MLLW&amp;interval=h&amp;action=other data here: https://en.wikipedia.org/wiki/1959_Escuminac_disaster#cite_note-mwr-1</t>
+  </si>
+  <si>
+    <t>ID_94</t>
+  </si>
+  <si>
+    <t>AL051959</t>
+  </si>
+  <si>
+    <t>Debra</t>
+  </si>
+  <si>
+    <t>Jul 23-28</t>
+  </si>
+  <si>
+    <t>ID_95</t>
+  </si>
+  <si>
+    <t>AL081959</t>
+  </si>
+  <si>
+    <t>Gracie</t>
+  </si>
+  <si>
+    <t>Sep 20 - Oct 2</t>
+  </si>
+  <si>
+    <t>ID_96</t>
+  </si>
+  <si>
+    <t>AL011960</t>
+  </si>
+  <si>
+    <t>Not Named 1960</t>
+  </si>
+  <si>
+    <t>Jun 22-29</t>
+  </si>
+  <si>
+    <t>MLW info gotten here chrome-extension://oemmndcbldboiebfnladdacbdfmadadm/https://www.aoml.noaa.gov/general/lib/lib1/nhclib/mwreviews/1960.pdf</t>
+  </si>
+  <si>
+    <t>ID_97</t>
+  </si>
+  <si>
+    <t>AL031960</t>
+  </si>
+  <si>
+    <t>Brenda</t>
+  </si>
+  <si>
     <t>gauge data from st. Petersburg: https://tidesandcurrents.noaa.gov/stationhome.html?id=8726520 other data here: https://en.wikipedia.org/wiki/1959_Escuminac_disaster#cite_note-mwr-1</t>
-  </si>
-  <si>
-    <t>ID_94</t>
-  </si>
-  <si>
-    <t>AL051959</t>
-  </si>
-  <si>
-    <t>Debra</t>
-  </si>
-  <si>
-    <t>Jul 23-28</t>
-  </si>
-  <si>
-    <t>ID_95</t>
-  </si>
-  <si>
-    <t>AL081959</t>
-  </si>
-  <si>
-    <t>Gracie</t>
-  </si>
-  <si>
-    <t>Sep 20 - Oct 2</t>
-  </si>
-  <si>
-    <t>ID_96</t>
-  </si>
-  <si>
-    <t>AL011960</t>
-  </si>
-  <si>
-    <t>Not Named 1960</t>
-  </si>
-  <si>
-    <t>Jun 22-29</t>
-  </si>
-  <si>
-    <t>MLW info gotten here chrome-extension://oemmndcbldboiebfnladdacbdfmadadm/https://www.aoml.noaa.gov/general/lib/lib1/nhclib/mwreviews/1960.pdf</t>
-  </si>
-  <si>
-    <t>ID_97</t>
-  </si>
-  <si>
-    <t>AL031960</t>
-  </si>
-  <si>
-    <t>Brenda</t>
   </si>
   <si>
     <t>ID_98</t>
@@ -7365,6 +7371,9 @@
       <c r="H77" s="2">
         <v>19628.666666666672</v>
       </c>
+      <c r="I77" t="s">
+        <v>324</v>
+      </c>
       <c r="J77">
         <v>1.524</v>
       </c>
@@ -7387,21 +7396,21 @@
         <v>19630</v>
       </c>
       <c r="S77" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="T77" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="78" spans="1:21">
       <c r="A78" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B78" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C78" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D78">
         <v>1954</v>
@@ -7443,18 +7452,18 @@
         <v>52</v>
       </c>
       <c r="U78" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="79" spans="1:21">
       <c r="A79" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B79" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C79" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D79">
         <v>1954</v>
@@ -7493,7 +7502,7 @@
         <v>19967</v>
       </c>
       <c r="S79" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="T79" t="s">
         <v>26</v>
@@ -7501,19 +7510,19 @@
     </row>
     <row r="80" spans="1:21">
       <c r="A80" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B80" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C80" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D80">
         <v>1954</v>
       </c>
       <c r="E80" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F80">
         <v>41.7</v>
@@ -7541,21 +7550,21 @@
         <v>-70.300161286068601</v>
       </c>
       <c r="T80" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U80" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="81" spans="1:21">
       <c r="A81" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B81" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C81" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D81">
         <v>1954</v>
@@ -7593,13 +7602,13 @@
     </row>
     <row r="82" spans="1:21">
       <c r="A82" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B82" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C82" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D82">
         <v>1955</v>
@@ -7643,13 +7652,13 @@
     </row>
     <row r="83" spans="1:21">
       <c r="A83" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B83" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C83" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D83">
         <v>1955</v>
@@ -7689,24 +7698,24 @@
         <v>20322</v>
       </c>
       <c r="S83" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="T83" t="s">
         <v>26</v>
       </c>
       <c r="U83" s="22" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="84" spans="1:21">
       <c r="A84" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B84" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C84" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D84">
         <v>1955</v>
@@ -7725,6 +7734,12 @@
       </c>
       <c r="I84" t="s">
         <v>61</v>
+      </c>
+      <c r="J84">
+        <v>0</v>
+      </c>
+      <c r="K84">
+        <v>0</v>
       </c>
       <c r="L84">
         <v>1.01</v>
@@ -7749,24 +7764,24 @@
         <v>20322</v>
       </c>
       <c r="S84" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="T84" t="s">
         <v>230</v>
       </c>
       <c r="U84" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="85" spans="1:21">
       <c r="A85" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B85" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C85" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D85">
         <v>1955</v>
@@ -7809,24 +7824,24 @@
         <v>20356</v>
       </c>
       <c r="S85" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="T85" t="s">
         <v>26</v>
       </c>
       <c r="U85" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="86" spans="1:21">
       <c r="A86" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B86" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C86" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D86">
         <v>1956</v>
@@ -7868,7 +7883,7 @@
         <v>20728</v>
       </c>
       <c r="S86" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="T86" t="s">
         <v>26</v>
@@ -7876,13 +7891,13 @@
     </row>
     <row r="87" spans="1:21">
       <c r="A87" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B87" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C87" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D87">
         <v>1957</v>
@@ -7924,7 +7939,7 @@
         <v>21000</v>
       </c>
       <c r="S87" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="T87" t="s">
         <v>26</v>
@@ -7932,13 +7947,13 @@
     </row>
     <row r="88" spans="1:21">
       <c r="A88" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B88" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C88" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D88">
         <v>1957</v>
@@ -7954,6 +7969,9 @@
       </c>
       <c r="H88" s="2">
         <v>21081.5</v>
+      </c>
+      <c r="I88" t="s">
+        <v>324</v>
       </c>
       <c r="J88">
         <v>1.0668</v>
@@ -7978,24 +7996,24 @@
         <v>21082</v>
       </c>
       <c r="S88" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="T88" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U88" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="89" spans="1:21">
       <c r="A89" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B89" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C89" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D89">
         <v>1958</v>
@@ -8037,7 +8055,7 @@
         <v>21456</v>
       </c>
       <c r="S89" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="T89" t="s">
         <v>26</v>
@@ -8045,13 +8063,13 @@
     </row>
     <row r="90" spans="1:21">
       <c r="A90" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B90" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C90" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D90">
         <v>1959</v>
@@ -8090,7 +8108,7 @@
         <v>21703</v>
       </c>
       <c r="S90" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="T90" t="s">
         <v>26</v>
@@ -8098,13 +8116,13 @@
     </row>
     <row r="91" spans="1:21">
       <c r="A91" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B91" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C91" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D91">
         <v>1959</v>
@@ -8150,18 +8168,18 @@
         <v>230</v>
       </c>
       <c r="U91" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="92" spans="1:21">
       <c r="A92" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B92" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C92" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D92">
         <v>1959</v>
@@ -8203,7 +8221,7 @@
         <v>21759</v>
       </c>
       <c r="S92" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="T92" t="s">
         <v>26</v>
@@ -8211,13 +8229,13 @@
     </row>
     <row r="93" spans="1:21">
       <c r="A93" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B93" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C93" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D93">
         <v>1959</v>
@@ -8259,7 +8277,7 @@
         <v>21825</v>
       </c>
       <c r="S93" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="T93" t="s">
         <v>26</v>
@@ -8267,13 +8285,13 @@
     </row>
     <row r="94" spans="1:21">
       <c r="A94" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B94" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C94" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D94">
         <v>1960</v>
@@ -8315,24 +8333,24 @@
         <v>22096</v>
       </c>
       <c r="S94" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="T94" t="s">
         <v>26</v>
       </c>
       <c r="U94" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="95" spans="1:21">
       <c r="A95" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B95" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C95" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D95">
         <v>1960</v>
@@ -8378,18 +8396,18 @@
         <v>52</v>
       </c>
       <c r="U95" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
     </row>
     <row r="96" spans="1:21">
       <c r="A96" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B96" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C96" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D96">
         <v>1960</v>
@@ -8428,7 +8446,7 @@
         <v>22173</v>
       </c>
       <c r="S96" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="T96" t="s">
         <v>26</v>
@@ -8436,13 +8454,13 @@
     </row>
     <row r="97" spans="1:21">
       <c r="A97" t="s">
+        <v>402</v>
+      </c>
+      <c r="B97" t="s">
+        <v>399</v>
+      </c>
+      <c r="C97" t="s">
         <v>400</v>
-      </c>
-      <c r="B97" t="s">
-        <v>397</v>
-      </c>
-      <c r="C97" t="s">
-        <v>398</v>
       </c>
       <c r="D97">
         <v>1960</v>
@@ -8487,7 +8505,7 @@
         <v>22172</v>
       </c>
       <c r="S97" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="T97" t="s">
         <v>26</v>
@@ -8495,13 +8513,13 @@
     </row>
     <row r="98" spans="1:21">
       <c r="A98" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B98" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C98" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D98">
         <v>1960</v>
@@ -8540,7 +8558,7 @@
         <v>22172</v>
       </c>
       <c r="S98" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="T98" t="s">
         <v>26</v>
@@ -8548,13 +8566,13 @@
     </row>
     <row r="99" spans="1:21">
       <c r="A99" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B99" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="C99" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D99">
         <v>1960</v>
@@ -8596,7 +8614,7 @@
         <v>22176</v>
       </c>
       <c r="S99" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="T99" t="s">
         <v>26</v>
@@ -8604,13 +8622,13 @@
     </row>
     <row r="100" spans="1:21">
       <c r="A100" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B100" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C100" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D100">
         <v>1961</v>
@@ -8652,7 +8670,7 @@
         <v>22540</v>
       </c>
       <c r="S100" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="T100" t="s">
         <v>26</v>
@@ -8660,19 +8678,19 @@
     </row>
     <row r="101" spans="1:21">
       <c r="A101" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B101" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="C101" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D101">
         <v>1961</v>
       </c>
       <c r="E101" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F101">
         <v>40.937199999999997</v>
@@ -8712,18 +8730,18 @@
         <v>230</v>
       </c>
       <c r="U101" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="102" spans="1:21">
       <c r="A102" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B102" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C102" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D102">
         <v>1962</v>
@@ -8740,10 +8758,13 @@
       <c r="H102" s="2">
         <v>22886.354166666672</v>
       </c>
-      <c r="J102">
+      <c r="I102" t="s">
+        <v>324</v>
+      </c>
+      <c r="L102">
         <v>0.91439999999999999</v>
       </c>
-      <c r="K102">
+      <c r="M102">
         <v>3</v>
       </c>
       <c r="N102">
@@ -8762,30 +8783,30 @@
         <v>22891</v>
       </c>
       <c r="S102" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="T102" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U102" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="103" spans="1:21">
       <c r="A103" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B103" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C103" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D103">
         <v>1962</v>
       </c>
       <c r="E103" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="F103">
         <v>43.605133333333328</v>
@@ -8808,18 +8829,18 @@
         <v>66</v>
       </c>
       <c r="U103" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
     </row>
     <row r="104" spans="1:21">
       <c r="A104" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B104" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="C104" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D104">
         <v>1963</v>
@@ -8858,7 +8879,7 @@
         <v>23274</v>
       </c>
       <c r="S104" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="T104" t="s">
         <v>26</v>
@@ -8866,13 +8887,13 @@
     </row>
     <row r="105" spans="1:21">
       <c r="A105" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B105" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C105" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D105">
         <v>1964</v>
@@ -8914,7 +8935,7 @@
         <v>23597</v>
       </c>
       <c r="S105" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="T105" t="s">
         <v>26</v>
@@ -8922,13 +8943,13 @@
     </row>
     <row r="106" spans="1:21">
       <c r="A106" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B106" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C106" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D106">
         <v>1964</v>
@@ -8945,10 +8966,13 @@
       <c r="H106" s="2">
         <v>23616.4375</v>
       </c>
-      <c r="J106">
+      <c r="I106" t="s">
+        <v>324</v>
+      </c>
+      <c r="L106">
         <v>1.8288</v>
       </c>
-      <c r="K106">
+      <c r="M106">
         <v>6</v>
       </c>
       <c r="N106">
@@ -8967,24 +8991,24 @@
         <v>23625</v>
       </c>
       <c r="S106" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="T106" s="11" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U106" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="107" spans="1:21">
       <c r="A107" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B107" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C107" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="D107">
         <v>1964</v>
@@ -9026,7 +9050,7 @@
         <v>23636</v>
       </c>
       <c r="S107" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="T107" t="s">
         <v>26</v>
@@ -9034,13 +9058,13 @@
     </row>
     <row r="108" spans="1:21">
       <c r="A108" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B108" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="C108" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="D108">
         <v>1964</v>
@@ -9082,7 +9106,7 @@
         <v>23655</v>
       </c>
       <c r="S108" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="T108" t="s">
         <v>26</v>
@@ -9090,13 +9114,13 @@
     </row>
     <row r="109" spans="1:21">
       <c r="A109" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B109" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C109" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="D109">
         <v>1964</v>
@@ -9138,7 +9162,7 @@
         <v>23666</v>
       </c>
       <c r="S109" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="T109" t="s">
         <v>26</v>
@@ -9146,13 +9170,13 @@
     </row>
     <row r="110" spans="1:21">
       <c r="A110" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B110" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C110" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D110">
         <v>1965</v>
@@ -9191,7 +9215,7 @@
         <v>23995</v>
       </c>
       <c r="S110" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="T110" t="s">
         <v>26</v>
@@ -9199,13 +9223,13 @@
     </row>
     <row r="111" spans="1:21">
       <c r="A111" t="s">
+        <v>455</v>
+      </c>
+      <c r="B111" t="s">
+        <v>452</v>
+      </c>
+      <c r="C111" t="s">
         <v>453</v>
-      </c>
-      <c r="B111" t="s">
-        <v>450</v>
-      </c>
-      <c r="C111" t="s">
-        <v>451</v>
       </c>
       <c r="D111">
         <v>1965</v>
@@ -9244,21 +9268,21 @@
         <v>23998</v>
       </c>
       <c r="S111" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="T111" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="112" spans="1:21">
       <c r="A112" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B112" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C112" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="D112">
         <v>1965</v>
@@ -9297,7 +9321,7 @@
         <v>24015</v>
       </c>
       <c r="S112" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="T112" t="s">
         <v>26</v>
@@ -9305,13 +9329,13 @@
     </row>
     <row r="113" spans="1:21">
       <c r="A113" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B113" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="C113" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D113">
         <v>1966</v>
@@ -9353,7 +9377,7 @@
         <v>24272</v>
       </c>
       <c r="S113" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="T113" s="7" t="s">
         <v>26</v>
@@ -9361,13 +9385,13 @@
     </row>
     <row r="114" spans="1:21">
       <c r="A114" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B114" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C114" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="D114">
         <v>1966</v>
@@ -9384,10 +9408,13 @@
       <c r="H114" s="2">
         <v>24384.729166666672</v>
       </c>
-      <c r="J114">
+      <c r="I114" t="s">
+        <v>324</v>
+      </c>
+      <c r="L114">
         <v>1.524</v>
       </c>
-      <c r="K114">
+      <c r="M114">
         <v>5</v>
       </c>
       <c r="N114">
@@ -9406,24 +9433,24 @@
         <v>24391</v>
       </c>
       <c r="S114" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="T114" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U114" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
     <row r="115" spans="1:21">
       <c r="A115" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B115" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="C115" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="D115">
         <v>1967</v>
@@ -9463,24 +9490,24 @@
         <v>24737</v>
       </c>
       <c r="S115" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="T115" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U115" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="116" spans="1:21">
       <c r="A116" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B116" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C116" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D116">
         <v>1968</v>
@@ -9519,7 +9546,7 @@
         <v>25002</v>
       </c>
       <c r="S116" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="T116" t="s">
         <v>26</v>
@@ -9527,13 +9554,13 @@
     </row>
     <row r="117" spans="1:21">
       <c r="A117" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B117" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="C117" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D117">
         <v>1968</v>
@@ -9550,6 +9577,9 @@
       <c r="H117" s="2">
         <v>25012.958333333328</v>
       </c>
+      <c r="I117" t="s">
+        <v>324</v>
+      </c>
       <c r="J117">
         <v>1.3715999999999999</v>
       </c>
@@ -9572,21 +9602,21 @@
         <v>25015</v>
       </c>
       <c r="S117" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="T117" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="118" spans="1:21">
       <c r="A118" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B118" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C118" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="D118">
         <v>1968</v>
@@ -9625,7 +9655,7 @@
         <v>25132</v>
       </c>
       <c r="S118" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="T118" t="s">
         <v>26</v>
@@ -9633,13 +9663,13 @@
     </row>
     <row r="119" spans="1:21">
       <c r="A119" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B119" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="C119" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D119">
         <v>1969</v>
@@ -9678,7 +9708,7 @@
         <v>25437</v>
       </c>
       <c r="S119" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="T119" t="s">
         <v>26</v>
@@ -9686,13 +9716,13 @@
     </row>
     <row r="120" spans="1:21">
       <c r="A120" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B120" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="C120" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D120">
         <v>1970</v>
@@ -9734,7 +9764,7 @@
         <v>25785</v>
       </c>
       <c r="S120" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="T120" t="s">
         <v>26</v>
@@ -9742,13 +9772,13 @@
     </row>
     <row r="121" spans="1:21">
       <c r="A121" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B121" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="C121" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="D121">
         <v>1971</v>
@@ -9765,10 +9795,13 @@
       <c r="H121" s="2">
         <v>26172.770833333328</v>
       </c>
-      <c r="J121">
+      <c r="I121" t="s">
+        <v>324</v>
+      </c>
+      <c r="L121">
         <v>0.60960000000000003</v>
       </c>
-      <c r="K121">
+      <c r="M121">
         <v>2</v>
       </c>
       <c r="N121">
@@ -9781,21 +9814,21 @@
         <v>-77.849999999999994</v>
       </c>
       <c r="T121" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U121" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="122" spans="1:21">
       <c r="A122" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B122" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="C122" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="D122">
         <v>1971</v>
@@ -9837,7 +9870,7 @@
         <v>26189</v>
       </c>
       <c r="S122" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="T122" t="s">
         <v>26</v>
@@ -9845,13 +9878,13 @@
     </row>
     <row r="123" spans="1:21">
       <c r="A123" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B123" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C123" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="D123">
         <v>1971</v>
@@ -9890,7 +9923,7 @@
         <v>26194</v>
       </c>
       <c r="S123" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="T123" t="s">
         <v>26</v>
@@ -9898,13 +9931,13 @@
     </row>
     <row r="124" spans="1:21">
       <c r="A124" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B124" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="C124" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="D124">
         <v>1971</v>
@@ -9921,10 +9954,13 @@
       <c r="H124" s="2">
         <v>26206.958333333328</v>
       </c>
-      <c r="J124">
+      <c r="I124" t="s">
+        <v>324</v>
+      </c>
+      <c r="L124">
         <v>2.13</v>
       </c>
-      <c r="K124">
+      <c r="M124">
         <v>7</v>
       </c>
       <c r="N124" s="7">
@@ -9938,21 +9974,21 @@
         <v>-75.905813467612802</v>
       </c>
       <c r="T124" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U124" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="125" spans="1:21">
       <c r="A125" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B125" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="C125" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="D125">
         <v>1972</v>
@@ -9991,24 +10027,24 @@
         <v>26473</v>
       </c>
       <c r="S125" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="T125" t="s">
         <v>26</v>
       </c>
       <c r="U125" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="126" spans="1:21">
       <c r="A126" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B126" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="C126" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="D126">
         <v>1972</v>
@@ -10025,10 +10061,13 @@
       <c r="H126" s="2">
         <v>26472.8125</v>
       </c>
-      <c r="J126">
+      <c r="I126" t="s">
+        <v>324</v>
+      </c>
+      <c r="L126">
         <v>0.94488000000000005</v>
       </c>
-      <c r="K126">
+      <c r="M126">
         <v>3.1</v>
       </c>
       <c r="N126">
@@ -10047,30 +10086,30 @@
         <v>26472</v>
       </c>
       <c r="S126" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="T126" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U126" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="127" spans="1:21">
       <c r="A127" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B127" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="C127" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D127">
         <v>1972</v>
       </c>
       <c r="E127" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F127">
         <v>44.638300000000001</v>
@@ -10110,18 +10149,18 @@
         <v>230</v>
       </c>
       <c r="U127" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="128" spans="1:21">
       <c r="A128" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B128" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="C128" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="D128">
         <v>1973</v>
@@ -10171,13 +10210,13 @@
     </row>
     <row r="129" spans="1:21">
       <c r="A129" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B129" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="C129" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D129">
         <v>1974</v>
@@ -10223,18 +10262,18 @@
         <v>230</v>
       </c>
       <c r="U129" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="130" spans="1:21">
       <c r="A130" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B130" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="C130" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="D130">
         <v>1974</v>
@@ -10284,13 +10323,13 @@
     </row>
     <row r="131" spans="1:21">
       <c r="A131" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B131" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="C131" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D131">
         <v>1975</v>
@@ -10332,7 +10371,7 @@
         <v>27661</v>
       </c>
       <c r="S131" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="T131" t="s">
         <v>26</v>
@@ -10340,13 +10379,13 @@
     </row>
     <row r="132" spans="1:21">
       <c r="A132" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B132" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="C132" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D132">
         <v>1976</v>
@@ -10394,24 +10433,24 @@
         <v>27981</v>
       </c>
       <c r="S132" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="T132" t="s">
         <v>26</v>
       </c>
       <c r="U132" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="133" spans="1:21">
       <c r="A133" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B133" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="C133" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D133">
         <v>1977</v>
@@ -10453,7 +10492,7 @@
         <v>28377</v>
       </c>
       <c r="S133" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="T133" t="s">
         <v>26</v>
@@ -10461,13 +10500,13 @@
     </row>
     <row r="134" spans="1:21">
       <c r="A134" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B134" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C134" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D134">
         <v>1978</v>
@@ -10507,18 +10546,18 @@
         <v>230</v>
       </c>
       <c r="U134" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="135" spans="1:21">
       <c r="A135" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B135" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="C135" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="D135">
         <v>1979</v>
@@ -10560,7 +10599,7 @@
         <v>29052</v>
       </c>
       <c r="S135" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="T135" t="s">
         <v>26</v>
@@ -10568,13 +10607,13 @@
     </row>
     <row r="136" spans="1:21">
       <c r="A136" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B136" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="C136" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="D136">
         <v>1979</v>
@@ -10616,7 +10655,7 @@
         <v>29065</v>
       </c>
       <c r="S136" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="T136" t="s">
         <v>26</v>
@@ -10624,13 +10663,13 @@
     </row>
     <row r="137" spans="1:21">
       <c r="A137" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B137" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="C137" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="D137">
         <v>1979</v>
@@ -10672,7 +10711,7 @@
         <v>29100</v>
       </c>
       <c r="S137" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="T137" t="s">
         <v>26</v>
@@ -10680,13 +10719,13 @@
     </row>
     <row r="138" spans="1:21">
       <c r="A138" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B138" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="C138" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="D138">
         <v>1979</v>
@@ -10703,10 +10742,13 @@
       <c r="H138" s="2">
         <v>29101.708333333328</v>
       </c>
-      <c r="J138">
+      <c r="I138" t="s">
+        <v>324</v>
+      </c>
+      <c r="L138">
         <v>1.2192000000000001</v>
       </c>
-      <c r="K138">
+      <c r="M138">
         <v>4</v>
       </c>
       <c r="N138" s="7">
@@ -10726,24 +10768,24 @@
         <v>29106</v>
       </c>
       <c r="S138" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="T138" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U138" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="139" spans="1:21">
       <c r="A139" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B139" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="C139" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="D139">
         <v>1979</v>
@@ -10785,7 +10827,7 @@
         <v>29105</v>
       </c>
       <c r="S139" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="T139" t="s">
         <v>26</v>
@@ -10793,13 +10835,13 @@
     </row>
     <row r="140" spans="1:21">
       <c r="A140" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="B140" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="C140" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="D140">
         <v>1979</v>
@@ -10841,7 +10883,7 @@
         <v>29113</v>
       </c>
       <c r="S140" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="T140" t="s">
         <v>26</v>
@@ -10849,13 +10891,13 @@
     </row>
     <row r="141" spans="1:21">
       <c r="A141" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="B141" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C141" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D141">
         <v>1980</v>
@@ -10897,7 +10939,7 @@
         <v>29444</v>
       </c>
       <c r="S141" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="T141" t="s">
         <v>26</v>
@@ -10905,13 +10947,13 @@
     </row>
     <row r="142" spans="1:21">
       <c r="A142" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="B142" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C142" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="D142">
         <v>1981</v>
@@ -10957,18 +10999,18 @@
         <v>230</v>
       </c>
       <c r="U142" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="143" spans="1:21">
       <c r="A143" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B143" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C143" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="D143">
         <v>1982</v>
@@ -11014,18 +11056,18 @@
         <v>230</v>
       </c>
       <c r="U143" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="144" spans="1:21">
       <c r="A144" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="B144" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="C144" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="D144">
         <v>1982</v>
@@ -11068,24 +11110,24 @@
         <v>30206</v>
       </c>
       <c r="S144" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="T144" t="s">
         <v>26</v>
       </c>
       <c r="U144" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="145" spans="1:21">
       <c r="A145" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B145" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="C145" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D145">
         <v>1983</v>
@@ -11127,7 +11169,7 @@
         <v>30549</v>
       </c>
       <c r="S145" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="T145" t="s">
         <v>26</v>
@@ -11135,13 +11177,13 @@
     </row>
     <row r="146" spans="1:21">
       <c r="A146" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="B146" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="C146" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="D146">
         <v>1984</v>
@@ -11158,10 +11200,13 @@
       <c r="H146" s="2">
         <v>30938.333333333328</v>
       </c>
-      <c r="J146">
+      <c r="I146" t="s">
+        <v>324</v>
+      </c>
+      <c r="L146">
         <v>1.7</v>
       </c>
-      <c r="K146">
+      <c r="M146">
         <v>5.5774299999999997</v>
       </c>
       <c r="N146">
@@ -11180,24 +11225,24 @@
         <v>30941</v>
       </c>
       <c r="S146" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="T146" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U146" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="147" spans="1:21">
       <c r="A147" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="B147" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C147" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="D147">
         <v>1984</v>
@@ -11243,18 +11288,18 @@
         <v>230</v>
       </c>
       <c r="U147" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="148" spans="1:21">
       <c r="A148" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="B148" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="C148" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="D148">
         <v>1985</v>
@@ -11271,10 +11316,13 @@
       <c r="H148" s="2">
         <v>31253.145833333328</v>
       </c>
-      <c r="J148">
+      <c r="I148" t="s">
+        <v>324</v>
+      </c>
+      <c r="L148">
         <v>0.5</v>
       </c>
-      <c r="K148">
+      <c r="M148">
         <v>1.64042</v>
       </c>
       <c r="N148">
@@ -11293,24 +11341,24 @@
         <v>31254</v>
       </c>
       <c r="S148" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="T148" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U148" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="149" spans="1:21">
       <c r="A149" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="B149" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="C149" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="D149">
         <v>1985</v>
@@ -11358,18 +11406,18 @@
         <v>26</v>
       </c>
       <c r="U149" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="150" spans="1:21">
       <c r="A150" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="B150" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="C150" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="D150">
         <v>1985</v>
@@ -11408,21 +11456,21 @@
         <v>31294</v>
       </c>
       <c r="S150" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="T150" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="151" spans="1:21">
       <c r="A151" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="B151" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="C151" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="D151">
         <v>1985</v>
@@ -11439,7 +11487,10 @@
       <c r="H151" s="2">
         <v>31317.25</v>
       </c>
-      <c r="J151">
+      <c r="I151" t="s">
+        <v>324</v>
+      </c>
+      <c r="L151">
         <v>1.8</v>
       </c>
       <c r="N151" s="7">
@@ -11459,24 +11510,24 @@
         <v>31322</v>
       </c>
       <c r="S151" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="T151" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U151" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="152" spans="1:21">
       <c r="A152" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B152" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="C152" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="D152">
         <v>1985</v>
@@ -11493,6 +11544,9 @@
       <c r="H152" s="2">
         <v>31317.6875</v>
       </c>
+      <c r="I152" t="s">
+        <v>324</v>
+      </c>
       <c r="J152">
         <v>2.1</v>
       </c>
@@ -11515,21 +11569,21 @@
         <v>31322</v>
       </c>
       <c r="S152" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="T152" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="153" spans="1:21">
       <c r="A153" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="B153" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="C153" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="D153">
         <v>1985</v>
@@ -11568,21 +11622,21 @@
         <v>31352</v>
       </c>
       <c r="S153" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="T153" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="154" spans="1:21">
       <c r="A154" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B154" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="C154" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="D154">
         <v>1985</v>
@@ -11621,21 +11675,21 @@
         <v>31374</v>
       </c>
       <c r="S154" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="T154" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="155" spans="1:21">
       <c r="A155" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B155" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C155" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="D155">
         <v>1986</v>
@@ -11652,6 +11706,9 @@
       <c r="H155" s="2">
         <v>31589.416666666672</v>
       </c>
+      <c r="I155" t="s">
+        <v>324</v>
+      </c>
       <c r="J155">
         <v>1.5849599999999999</v>
       </c>
@@ -11674,21 +11731,21 @@
         <v>31591</v>
       </c>
       <c r="S155" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="T155" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="156" spans="1:21">
       <c r="A156" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="B156" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="C156" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="D156">
         <v>1986</v>
@@ -11730,7 +11787,7 @@
         <v>31654</v>
       </c>
       <c r="S156" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="T156" t="s">
         <v>26</v>
@@ -11738,13 +11795,13 @@
     </row>
     <row r="157" spans="1:21">
       <c r="A157" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="B157" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C157" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D157">
         <v>1987</v>
@@ -11784,18 +11841,18 @@
         <v>230</v>
       </c>
       <c r="U157" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="158" spans="1:21">
       <c r="A158" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="B158" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="C158" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="D158">
         <v>1987</v>
@@ -11834,21 +11891,21 @@
         <v>32064</v>
       </c>
       <c r="S158" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="T158" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="159" spans="1:21">
       <c r="A159" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B159" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="C159" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="D159">
         <v>1988</v>
@@ -11887,21 +11944,21 @@
         <v>32365</v>
       </c>
       <c r="S159" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="T159" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="160" spans="1:21">
       <c r="A160" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="B160" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="C160" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="D160">
         <v>1988</v>
@@ -11941,21 +11998,21 @@
         <v>32384</v>
       </c>
       <c r="S160" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="T160" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U160" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="161" spans="1:21">
       <c r="A161" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="B161" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="C161" t="s">
         <v>323</v>
@@ -12000,7 +12057,7 @@
         <v>32397</v>
       </c>
       <c r="S161" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="T161" t="s">
         <v>26</v>
@@ -12008,13 +12065,13 @@
     </row>
     <row r="162" spans="1:21">
       <c r="A162" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="B162" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="C162" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="D162">
         <v>1988</v>
@@ -12032,7 +12089,7 @@
         <v>32402.875</v>
       </c>
       <c r="J162" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="K162">
         <v>6</v>
@@ -12053,21 +12110,21 @@
         <v>32406</v>
       </c>
       <c r="S162" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="T162" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="163" spans="1:21">
       <c r="A163" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="B163" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="C163" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="D163">
         <v>1988</v>
@@ -12106,21 +12163,21 @@
         <v>32473</v>
       </c>
       <c r="S163" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="T163" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="164" spans="1:21">
       <c r="A164" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="B164" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="C164" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="D164">
         <v>1989</v>
@@ -12160,24 +12217,24 @@
         <v>32690</v>
       </c>
       <c r="S164" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="T164" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U164" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="165" spans="1:21">
       <c r="A165" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="B165" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="C165" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="D165">
         <v>1989</v>
@@ -12219,7 +12276,7 @@
         <v>32723</v>
       </c>
       <c r="S165" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="T165" t="s">
         <v>26</v>
@@ -12227,13 +12284,13 @@
     </row>
     <row r="166" spans="1:21">
       <c r="A166" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B166" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="C166" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="D166">
         <v>1989</v>
@@ -12275,7 +12332,7 @@
         <v>32773</v>
       </c>
       <c r="S166" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="T166" t="s">
         <v>26</v>
@@ -12283,13 +12340,13 @@
     </row>
     <row r="167" spans="1:21">
       <c r="A167" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="B167" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="C167" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="D167">
         <v>1989</v>
@@ -12328,7 +12385,7 @@
         <v>32797</v>
       </c>
       <c r="S167" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="T167" t="s">
         <v>26</v>
@@ -12336,13 +12393,13 @@
     </row>
     <row r="168" spans="1:21">
       <c r="A168" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="B168" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="C168" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="D168">
         <v>1990</v>
@@ -12382,30 +12439,30 @@
         <v>33159</v>
       </c>
       <c r="S168" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="T168" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U168" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="169" spans="1:21">
       <c r="A169" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B169" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="C169" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="D169">
         <v>1991</v>
       </c>
       <c r="E169" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="F169">
         <v>41.815399999999997</v>
@@ -12441,7 +12498,7 @@
         <v>33479</v>
       </c>
       <c r="S169" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="T169" t="s">
         <v>26</v>
@@ -12449,13 +12506,13 @@
     </row>
     <row r="170" spans="1:21">
       <c r="A170" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="B170" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="C170" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="D170">
         <v>1992</v>
@@ -12497,7 +12554,7 @@
         <v>33844</v>
       </c>
       <c r="S170" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="T170" t="s">
         <v>26</v>
@@ -12505,13 +12562,13 @@
     </row>
     <row r="171" spans="1:21">
       <c r="A171" t="s">
+        <v>690</v>
+      </c>
+      <c r="B171" t="s">
+        <v>687</v>
+      </c>
+      <c r="C171" t="s">
         <v>688</v>
-      </c>
-      <c r="B171" t="s">
-        <v>685</v>
-      </c>
-      <c r="C171" t="s">
-        <v>686</v>
       </c>
       <c r="D171">
         <v>1992</v>
@@ -12553,7 +12610,7 @@
         <v>33844</v>
       </c>
       <c r="S171" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="T171" t="s">
         <v>26</v>
@@ -12561,13 +12618,13 @@
     </row>
     <row r="172" spans="1:21">
       <c r="A172" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="B172" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="C172" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D172">
         <v>1993</v>
@@ -12615,7 +12672,7 @@
         <v>34141</v>
       </c>
       <c r="S172" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="T172" t="s">
         <v>26</v>
@@ -12623,13 +12680,13 @@
     </row>
     <row r="173" spans="1:21">
       <c r="A173" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="B173" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="C173" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="D173">
         <v>1993</v>
@@ -12646,11 +12703,13 @@
       <c r="H173" s="2">
         <v>34212.9375</v>
       </c>
-      <c r="I173" s="19"/>
-      <c r="J173">
+      <c r="I173" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="L173">
         <v>3.11</v>
       </c>
-      <c r="K173">
+      <c r="M173">
         <v>10.199999999999999</v>
       </c>
       <c r="N173">
@@ -12669,24 +12728,24 @@
         <v>34213</v>
       </c>
       <c r="S173" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="T173" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
       <c r="U173" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="174" spans="1:21">
       <c r="A174" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B174" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="C174" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="D174">
         <v>1994</v>
@@ -12725,7 +12784,7 @@
         <v>34522</v>
       </c>
       <c r="S174" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="T174" t="s">
         <v>26</v>
@@ -12733,13 +12792,13 @@
     </row>
     <row r="175" spans="1:21">
       <c r="A175" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B175" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="C175" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="D175">
         <v>1994</v>
@@ -12779,24 +12838,24 @@
         <v>34565</v>
       </c>
       <c r="S175" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="T175" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U175" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="176" spans="1:21" ht="15.75">
       <c r="A176" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="B176" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="C176" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="D176">
         <v>1994</v>
@@ -12836,24 +12895,24 @@
         <v>34659</v>
       </c>
       <c r="S176" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="T176" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U176" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="177" spans="1:21">
       <c r="A177" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B177" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="C177" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="D177">
         <v>1995</v>
@@ -12892,21 +12951,21 @@
         <v>34861</v>
       </c>
       <c r="S177" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="T177" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="178" spans="1:21">
       <c r="A178" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B178" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="C178" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="D178">
         <v>1995</v>
@@ -12948,24 +13007,24 @@
         <v>34917</v>
       </c>
       <c r="S178" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="T178" t="s">
         <v>26</v>
       </c>
       <c r="U178" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
     </row>
     <row r="179" spans="1:21">
       <c r="A179" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="B179" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C179" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="D179">
         <v>1995</v>
@@ -13007,7 +13066,7 @@
         <v>34917</v>
       </c>
       <c r="S179" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="T179" t="s">
         <v>26</v>
@@ -13015,13 +13074,13 @@
     </row>
     <row r="180" spans="1:21">
       <c r="A180" t="s">
+        <v>723</v>
+      </c>
+      <c r="B180" t="s">
         <v>721</v>
       </c>
-      <c r="B180" t="s">
-        <v>719</v>
-      </c>
       <c r="C180" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="D180">
         <v>1995</v>
@@ -13063,24 +13122,24 @@
         <v>34917</v>
       </c>
       <c r="S180" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="T180" t="s">
         <v>26</v>
       </c>
       <c r="U180" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
     </row>
     <row r="181" spans="1:21">
       <c r="A181" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="B181" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="C181" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="D181">
         <v>1995</v>
@@ -13097,10 +13156,13 @@
       <c r="H181" s="2">
         <v>34934.666666666664</v>
       </c>
-      <c r="J181">
+      <c r="I181" t="s">
+        <v>324</v>
+      </c>
+      <c r="L181">
         <v>0.61</v>
       </c>
-      <c r="K181">
+      <c r="M181">
         <v>2</v>
       </c>
       <c r="N181">
@@ -13119,24 +13181,24 @@
         <v>34939</v>
       </c>
       <c r="S181" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="T181" t="s">
         <v>26</v>
       </c>
       <c r="U181" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
     </row>
     <row r="182" spans="1:21">
       <c r="A182" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="B182" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="C182" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="D182">
         <v>1995</v>
@@ -13186,13 +13248,13 @@
     </row>
     <row r="183" spans="1:21">
       <c r="A183" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B183" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="C183" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="D183">
         <v>1996</v>
@@ -13231,24 +13293,24 @@
         <v>35260</v>
       </c>
       <c r="S183" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="T183" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U183" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
     </row>
     <row r="184" spans="1:21">
       <c r="A184" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="B184" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="C184" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="D184">
         <v>1996</v>
@@ -13289,13 +13351,13 @@
     </row>
     <row r="185" spans="1:21">
       <c r="A185" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="B185" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="C185" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="D185">
         <v>1996</v>
@@ -13337,7 +13399,7 @@
         <v>35346</v>
       </c>
       <c r="S185" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="T185" t="s">
         <v>26</v>
@@ -13345,13 +13407,13 @@
     </row>
     <row r="186" spans="1:21">
       <c r="A186" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="B186" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="C186" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="D186">
         <v>1997</v>
@@ -13393,7 +13455,7 @@
         <v>35638</v>
       </c>
       <c r="S186" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="T186" t="s">
         <v>26</v>
@@ -13401,13 +13463,13 @@
     </row>
     <row r="187" spans="1:21">
       <c r="A187" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="B187" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="C187" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="D187">
         <v>1998</v>
@@ -13446,21 +13508,21 @@
         <v>36031</v>
       </c>
       <c r="S187" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="T187" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="188" spans="1:21">
       <c r="A188" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="B188" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="C188" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="D188">
         <v>1998</v>
@@ -13501,13 +13563,13 @@
     </row>
     <row r="189" spans="1:21">
       <c r="A189" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="B189" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="C189" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="D189">
         <v>1998</v>
@@ -13546,24 +13608,24 @@
         <v>36046</v>
       </c>
       <c r="S189" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="T189" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U189" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
     </row>
     <row r="190" spans="1:21">
       <c r="A190" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="B190" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="C190" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="D190">
         <v>1998</v>
@@ -13605,7 +13667,7 @@
         <v>36051</v>
       </c>
       <c r="S190" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="T190" t="s">
         <v>26</v>
@@ -13613,13 +13675,13 @@
     </row>
     <row r="191" spans="1:21">
       <c r="A191" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="B191" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C191" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="D191">
         <v>1998</v>
@@ -13658,7 +13720,7 @@
         <v>36069</v>
       </c>
       <c r="S191" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="T191" t="s">
         <v>26</v>
@@ -13666,13 +13728,13 @@
     </row>
     <row r="192" spans="1:21">
       <c r="A192" t="s">
+        <v>765</v>
+      </c>
+      <c r="B192" t="s">
+        <v>762</v>
+      </c>
+      <c r="C192" t="s">
         <v>763</v>
-      </c>
-      <c r="B192" t="s">
-        <v>760</v>
-      </c>
-      <c r="C192" t="s">
-        <v>761</v>
       </c>
       <c r="D192">
         <v>1998</v>
@@ -13711,7 +13773,7 @@
         <v>36069</v>
       </c>
       <c r="S192" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="T192" t="s">
         <v>26</v>
@@ -13719,13 +13781,13 @@
     </row>
     <row r="193" spans="1:21">
       <c r="A193" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="B193" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="C193" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="D193">
         <v>1998</v>
@@ -13767,7 +13829,7 @@
         <v>36108</v>
       </c>
       <c r="S193" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="T193" t="s">
         <v>26</v>
@@ -13775,13 +13837,13 @@
     </row>
     <row r="194" spans="1:21">
       <c r="A194" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="B194" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="C194" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="D194">
         <v>1999</v>
@@ -13820,7 +13882,7 @@
         <v>36397</v>
       </c>
       <c r="S194" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="T194" t="s">
         <v>26</v>
@@ -13828,13 +13890,13 @@
     </row>
     <row r="195" spans="1:21">
       <c r="A195" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="B195" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="C195" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="D195">
         <v>1999</v>
@@ -13876,24 +13938,24 @@
         <v>36411</v>
       </c>
       <c r="S195" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="T195" t="s">
         <v>26</v>
       </c>
       <c r="U195" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
     </row>
     <row r="196" spans="1:21">
       <c r="A196" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="B196" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="C196" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="D196">
         <v>1999</v>
@@ -13938,7 +14000,7 @@
         <v>36422</v>
       </c>
       <c r="S196" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="T196" t="s">
         <v>26</v>
@@ -13946,13 +14008,13 @@
     </row>
     <row r="197" spans="1:21">
       <c r="A197" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="B197" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="C197" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="D197">
         <v>1999</v>
@@ -13994,7 +14056,7 @@
         <v>36425</v>
       </c>
       <c r="S197" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="T197" t="s">
         <v>26</v>
@@ -14002,13 +14064,13 @@
     </row>
     <row r="198" spans="1:21">
       <c r="A198" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="B198" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="C198" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="D198">
         <v>1999</v>
@@ -14048,24 +14110,24 @@
         <v>36452</v>
       </c>
       <c r="S198" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="T198" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U198" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="199" spans="1:21">
       <c r="A199" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="B199" t="s">
-        <v>788</v>
+        <v>790</v>
       </c>
       <c r="C199" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="D199">
         <v>2000</v>
@@ -14105,24 +14167,24 @@
         <v>36790</v>
       </c>
       <c r="S199" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="T199" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U199" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="200" spans="1:21">
       <c r="A200" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="B200" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="C200" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D200">
         <v>2000</v>
@@ -14162,24 +14224,24 @@
         <v>36794</v>
       </c>
       <c r="S200" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="T200" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U200" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="201" spans="1:21">
       <c r="A201" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="B201" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="C201" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="D201">
         <v>2001</v>
@@ -14219,24 +14281,24 @@
         <v>37061</v>
       </c>
       <c r="S201" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="T201" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U201" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="202" spans="1:21">
       <c r="A202" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="B202" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="C202" t="s">
-        <v>798</v>
+        <v>800</v>
       </c>
       <c r="D202">
         <v>2001</v>
@@ -14275,7 +14337,7 @@
         <v>37111</v>
       </c>
       <c r="S202" t="s">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="T202" t="s">
         <v>26</v>
@@ -14283,13 +14345,13 @@
     </row>
     <row r="203" spans="1:21">
       <c r="A203" t="s">
-        <v>800</v>
+        <v>802</v>
       </c>
       <c r="B203" t="s">
-        <v>801</v>
+        <v>803</v>
       </c>
       <c r="C203" t="s">
-        <v>802</v>
+        <v>804</v>
       </c>
       <c r="D203">
         <v>2001</v>
@@ -14328,21 +14390,21 @@
         <v>37155</v>
       </c>
       <c r="S203" t="s">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="T203" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="204" spans="1:21">
       <c r="A204" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="B204" t="s">
-        <v>805</v>
+        <v>807</v>
       </c>
       <c r="C204" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="D204">
         <v>2002</v>
@@ -14381,21 +14443,21 @@
         <v>37510</v>
       </c>
       <c r="S204" t="s">
-        <v>807</v>
+        <v>809</v>
       </c>
       <c r="T204" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="205" spans="1:21">
       <c r="A205" t="s">
-        <v>808</v>
+        <v>810</v>
       </c>
       <c r="B205" t="s">
-        <v>809</v>
+        <v>811</v>
       </c>
       <c r="C205" t="s">
-        <v>810</v>
+        <v>812</v>
       </c>
       <c r="D205">
         <v>2002</v>
@@ -14434,24 +14496,24 @@
         <v>37514</v>
       </c>
       <c r="S205" t="s">
-        <v>811</v>
+        <v>813</v>
       </c>
       <c r="T205" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U205" t="s">
-        <v>812</v>
+        <v>814</v>
       </c>
     </row>
     <row r="206" spans="1:21">
       <c r="A206" t="s">
-        <v>813</v>
+        <v>815</v>
       </c>
       <c r="B206" t="s">
-        <v>814</v>
+        <v>816</v>
       </c>
       <c r="C206" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="D206">
         <v>2002</v>
@@ -14493,7 +14555,7 @@
         <v>37514</v>
       </c>
       <c r="S206" t="s">
-        <v>816</v>
+        <v>818</v>
       </c>
       <c r="T206" t="s">
         <v>26</v>
@@ -14501,13 +14563,13 @@
     </row>
     <row r="207" spans="1:21">
       <c r="A207" t="s">
-        <v>817</v>
+        <v>819</v>
       </c>
       <c r="B207" t="s">
-        <v>818</v>
+        <v>820</v>
       </c>
       <c r="C207" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="D207">
         <v>2002</v>
@@ -14547,24 +14609,24 @@
         <v>37526</v>
       </c>
       <c r="S207" t="s">
-        <v>819</v>
+        <v>821</v>
       </c>
       <c r="T207" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U207" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="208" spans="1:21">
       <c r="A208" t="s">
-        <v>820</v>
+        <v>822</v>
       </c>
       <c r="B208" t="s">
-        <v>821</v>
+        <v>823</v>
       </c>
       <c r="C208" t="s">
-        <v>822</v>
+        <v>824</v>
       </c>
       <c r="D208">
         <v>2002</v>
@@ -14606,7 +14668,7 @@
         <v>37533</v>
       </c>
       <c r="S208" t="s">
-        <v>823</v>
+        <v>825</v>
       </c>
       <c r="T208" t="s">
         <v>26</v>
@@ -14614,13 +14676,13 @@
     </row>
     <row r="209" spans="1:21">
       <c r="A209" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="B209" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="C209" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="D209">
         <v>2002</v>
@@ -14659,21 +14721,21 @@
         <v>37541</v>
       </c>
       <c r="S209" t="s">
-        <v>827</v>
+        <v>829</v>
       </c>
       <c r="T209" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="210" spans="1:21">
       <c r="A210" t="s">
-        <v>828</v>
+        <v>830</v>
       </c>
       <c r="B210" t="s">
-        <v>829</v>
+        <v>831</v>
       </c>
       <c r="C210" t="s">
-        <v>830</v>
+        <v>832</v>
       </c>
       <c r="D210">
         <v>2003</v>
@@ -14713,21 +14775,21 @@
         <v>37805</v>
       </c>
       <c r="S210" t="s">
-        <v>831</v>
+        <v>833</v>
       </c>
       <c r="T210" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="211" spans="1:21">
       <c r="A211" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="B211" t="s">
-        <v>833</v>
+        <v>835</v>
       </c>
       <c r="C211" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="D211">
         <v>2003</v>
@@ -14769,24 +14831,24 @@
         <v>37819</v>
       </c>
       <c r="S211" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="T211" t="s">
         <v>26</v>
       </c>
       <c r="U211" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="212" spans="1:21">
       <c r="A212" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="B212" t="s">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="C212" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
       <c r="D212">
         <v>2003</v>
@@ -14825,21 +14887,21 @@
         <v>1364</v>
       </c>
       <c r="S212" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="T212" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="213" spans="1:21">
       <c r="A213" t="s">
-        <v>839</v>
+        <v>841</v>
       </c>
       <c r="B213" t="s">
-        <v>840</v>
+        <v>842</v>
       </c>
       <c r="C213" t="s">
-        <v>841</v>
+        <v>843</v>
       </c>
       <c r="D213">
         <v>2004</v>
@@ -14878,24 +14940,24 @@
         <v>38205</v>
       </c>
       <c r="S213" t="s">
-        <v>842</v>
+        <v>844</v>
       </c>
       <c r="T213" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U213" t="s">
-        <v>843</v>
+        <v>845</v>
       </c>
     </row>
     <row r="214" spans="1:21">
       <c r="A214" t="s">
-        <v>844</v>
+        <v>846</v>
       </c>
       <c r="B214" t="s">
-        <v>845</v>
+        <v>847</v>
       </c>
       <c r="C214" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="D214">
         <v>2004</v>
@@ -14937,7 +14999,7 @@
         <v>38214</v>
       </c>
       <c r="S214" t="s">
-        <v>846</v>
+        <v>848</v>
       </c>
       <c r="T214" t="s">
         <v>26</v>
@@ -14945,13 +15007,13 @@
     </row>
     <row r="215" spans="1:21">
       <c r="A215" t="s">
+        <v>849</v>
+      </c>
+      <c r="B215" t="s">
         <v>847</v>
       </c>
-      <c r="B215" t="s">
-        <v>845</v>
-      </c>
       <c r="C215" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="D215">
         <v>2004</v>
@@ -15002,24 +15064,24 @@
         <v>38214</v>
       </c>
       <c r="S215" t="s">
-        <v>848</v>
+        <v>850</v>
       </c>
       <c r="T215" t="s">
         <v>26</v>
       </c>
       <c r="U215" t="s">
-        <v>849</v>
+        <v>851</v>
       </c>
     </row>
     <row r="216" spans="1:21">
       <c r="A216" t="s">
-        <v>850</v>
+        <v>852</v>
       </c>
       <c r="B216" t="s">
-        <v>851</v>
+        <v>853</v>
       </c>
       <c r="C216" t="s">
-        <v>852</v>
+        <v>854</v>
       </c>
       <c r="D216">
         <v>2004</v>
@@ -15067,7 +15129,7 @@
         <v>38231</v>
       </c>
       <c r="S216" t="s">
-        <v>853</v>
+        <v>855</v>
       </c>
       <c r="T216" t="s">
         <v>26</v>
@@ -15075,13 +15137,13 @@
     </row>
     <row r="217" spans="1:21">
       <c r="A217" t="s">
-        <v>854</v>
+        <v>856</v>
       </c>
       <c r="B217" t="s">
-        <v>855</v>
+        <v>857</v>
       </c>
       <c r="C217" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="D217">
         <v>2004</v>
@@ -15129,24 +15191,24 @@
         <v>38240</v>
       </c>
       <c r="S217" t="s">
-        <v>856</v>
+        <v>858</v>
       </c>
       <c r="T217" t="s">
         <v>26</v>
       </c>
       <c r="U217" t="s">
-        <v>857</v>
+        <v>859</v>
       </c>
     </row>
     <row r="218" spans="1:21">
       <c r="A218" t="s">
-        <v>858</v>
+        <v>860</v>
       </c>
       <c r="B218" t="s">
-        <v>859</v>
+        <v>861</v>
       </c>
       <c r="C218" t="s">
-        <v>860</v>
+        <v>862</v>
       </c>
       <c r="D218">
         <v>2004</v>
@@ -15185,21 +15247,21 @@
         <v>38254</v>
       </c>
       <c r="S218" t="s">
-        <v>861</v>
+        <v>863</v>
       </c>
       <c r="T218" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="219" spans="1:21">
       <c r="A219" t="s">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="B219" t="s">
-        <v>863</v>
+        <v>865</v>
       </c>
       <c r="C219" t="s">
-        <v>864</v>
+        <v>866</v>
       </c>
       <c r="D219">
         <v>2004</v>
@@ -15244,7 +15306,7 @@
         <v>38259</v>
       </c>
       <c r="S219" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
       <c r="T219" t="s">
         <v>26</v>
@@ -15252,13 +15314,13 @@
     </row>
     <row r="220" spans="1:21">
       <c r="A220" t="s">
-        <v>866</v>
+        <v>868</v>
       </c>
       <c r="B220" t="s">
-        <v>867</v>
+        <v>869</v>
       </c>
       <c r="C220" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D220">
         <v>2005</v>
@@ -15298,24 +15360,24 @@
         <v>38544</v>
       </c>
       <c r="S220" t="s">
-        <v>868</v>
+        <v>870</v>
       </c>
       <c r="T220" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U220" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="221" spans="1:21">
       <c r="A221" t="s">
-        <v>869</v>
+        <v>871</v>
       </c>
       <c r="B221" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
       <c r="C221" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="D221">
         <v>2005</v>
@@ -15333,7 +15395,7 @@
         <v>38543.833333333343</v>
       </c>
       <c r="I221" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="L221">
         <v>3.2</v>
@@ -15357,7 +15419,7 @@
         <v>38551</v>
       </c>
       <c r="S221" t="s">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="T221" t="s">
         <v>26</v>
@@ -15365,13 +15427,13 @@
     </row>
     <row r="222" spans="1:21">
       <c r="A222" t="s">
-        <v>873</v>
+        <v>875</v>
       </c>
       <c r="B222" t="s">
-        <v>874</v>
+        <v>876</v>
       </c>
       <c r="C222" t="s">
-        <v>875</v>
+        <v>877</v>
       </c>
       <c r="D222">
         <v>2005</v>
@@ -15410,21 +15472,21 @@
         <v>38595</v>
       </c>
       <c r="S222" t="s">
-        <v>876</v>
+        <v>878</v>
       </c>
       <c r="T222" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="223" spans="1:21">
       <c r="A223" t="s">
-        <v>877</v>
+        <v>879</v>
       </c>
       <c r="B223" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="C223" t="s">
-        <v>879</v>
+        <v>881</v>
       </c>
       <c r="D223">
         <v>2005</v>
@@ -15464,24 +15526,24 @@
         <v>38612</v>
       </c>
       <c r="S223" t="s">
-        <v>880</v>
+        <v>882</v>
       </c>
       <c r="T223" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U223" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="224" spans="1:21">
       <c r="A224" t="s">
-        <v>881</v>
+        <v>883</v>
       </c>
       <c r="B224" t="s">
-        <v>882</v>
+        <v>884</v>
       </c>
       <c r="C224" t="s">
-        <v>883</v>
+        <v>885</v>
       </c>
       <c r="D224">
         <v>2005</v>
@@ -15499,7 +15561,7 @@
         <v>38619.354166666657</v>
       </c>
       <c r="I224" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="L224">
         <v>5.4</v>
@@ -15523,7 +15585,7 @@
         <v>38621</v>
       </c>
       <c r="S224" t="s">
-        <v>884</v>
+        <v>886</v>
       </c>
       <c r="T224" t="s">
         <v>26</v>
@@ -15531,13 +15593,13 @@
     </row>
     <row r="225" spans="1:21">
       <c r="A225" t="s">
-        <v>885</v>
+        <v>887</v>
       </c>
       <c r="B225" t="s">
-        <v>886</v>
+        <v>888</v>
       </c>
       <c r="C225" t="s">
-        <v>887</v>
+        <v>889</v>
       </c>
       <c r="D225">
         <v>2005</v>
@@ -15576,21 +15638,21 @@
         <v>38651</v>
       </c>
       <c r="S225" t="s">
-        <v>888</v>
+        <v>890</v>
       </c>
       <c r="T225" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="226" spans="1:21">
       <c r="A226" t="s">
-        <v>889</v>
+        <v>891</v>
       </c>
       <c r="B226" t="s">
-        <v>890</v>
+        <v>892</v>
       </c>
       <c r="C226" t="s">
-        <v>891</v>
+        <v>893</v>
       </c>
       <c r="D226">
         <v>2006</v>
@@ -15638,7 +15700,7 @@
         <v>38964</v>
       </c>
       <c r="S226" t="s">
-        <v>892</v>
+        <v>894</v>
       </c>
       <c r="T226" t="s">
         <v>26</v>
@@ -15646,13 +15708,13 @@
     </row>
     <row r="227" spans="1:21">
       <c r="A227" t="s">
-        <v>893</v>
+        <v>895</v>
       </c>
       <c r="B227" t="s">
-        <v>894</v>
+        <v>896</v>
       </c>
       <c r="C227" t="s">
-        <v>895</v>
+        <v>897</v>
       </c>
       <c r="D227">
         <v>2007</v>
@@ -15694,7 +15756,7 @@
         <v>39339</v>
       </c>
       <c r="S227" t="s">
-        <v>896</v>
+        <v>898</v>
       </c>
       <c r="T227" t="s">
         <v>26</v>
@@ -15702,13 +15764,13 @@
     </row>
     <row r="228" spans="1:21">
       <c r="A228" t="s">
-        <v>897</v>
+        <v>899</v>
       </c>
       <c r="B228" t="s">
-        <v>898</v>
+        <v>900</v>
       </c>
       <c r="C228" t="s">
-        <v>899</v>
+        <v>901</v>
       </c>
       <c r="D228">
         <v>2008</v>
@@ -15756,7 +15818,7 @@
         <v>39656</v>
       </c>
       <c r="S228" t="s">
-        <v>900</v>
+        <v>902</v>
       </c>
       <c r="T228" t="s">
         <v>26</v>
@@ -15764,13 +15826,13 @@
     </row>
     <row r="229" spans="1:21">
       <c r="A229" t="s">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="B229" t="s">
-        <v>902</v>
+        <v>904</v>
       </c>
       <c r="C229" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="D229">
         <v>2008</v>
@@ -15810,24 +15872,24 @@
         <v>39688</v>
       </c>
       <c r="S229" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="T229" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U229" s="20" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
     </row>
     <row r="230" spans="1:21">
       <c r="A230" t="s">
-        <v>905</v>
+        <v>907</v>
       </c>
       <c r="B230" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="C230" t="s">
-        <v>810</v>
+        <v>812</v>
       </c>
       <c r="D230">
         <v>2008</v>
@@ -15845,7 +15907,7 @@
         <v>39692.625</v>
       </c>
       <c r="I230" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="J230">
         <v>3.1089600000000002</v>
@@ -15875,7 +15937,7 @@
         <v>39696</v>
       </c>
       <c r="S230" t="s">
-        <v>907</v>
+        <v>909</v>
       </c>
       <c r="T230" t="s">
         <v>26</v>
@@ -15883,13 +15945,13 @@
     </row>
     <row r="231" spans="1:21">
       <c r="A231" t="s">
-        <v>908</v>
+        <v>910</v>
       </c>
       <c r="B231" t="s">
-        <v>909</v>
+        <v>911</v>
       </c>
       <c r="C231" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="D231">
         <v>2008</v>
@@ -15937,24 +15999,24 @@
         <v>39699</v>
       </c>
       <c r="S231" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="T231" t="s">
         <v>26</v>
       </c>
       <c r="U231" t="s">
-        <v>911</v>
+        <v>913</v>
       </c>
     </row>
     <row r="232" spans="1:21">
       <c r="A232" t="s">
-        <v>912</v>
+        <v>914</v>
       </c>
       <c r="B232" t="s">
-        <v>913</v>
+        <v>915</v>
       </c>
       <c r="C232" t="s">
-        <v>914</v>
+        <v>916</v>
       </c>
       <c r="D232">
         <v>2008</v>
@@ -15972,7 +16034,7 @@
         <v>39704.375</v>
       </c>
       <c r="I232" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="L232">
         <v>5.91</v>
@@ -15996,7 +16058,7 @@
         <v>39706</v>
       </c>
       <c r="S232" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="T232" t="s">
         <v>26</v>
@@ -16004,13 +16066,13 @@
     </row>
     <row r="233" spans="1:21">
       <c r="A233" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="B233" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="C233" t="s">
-        <v>841</v>
+        <v>843</v>
       </c>
       <c r="D233">
         <v>2010</v>
@@ -16052,18 +16114,18 @@
         <v>52</v>
       </c>
       <c r="U233" t="s">
-        <v>918</v>
+        <v>920</v>
       </c>
     </row>
     <row r="234" spans="1:21">
       <c r="A234" t="s">
-        <v>919</v>
+        <v>921</v>
       </c>
       <c r="B234" t="s">
-        <v>920</v>
+        <v>922</v>
       </c>
       <c r="C234" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="D234">
         <v>2010</v>
@@ -16103,24 +16165,24 @@
         <v>40427</v>
       </c>
       <c r="S234" t="s">
-        <v>921</v>
+        <v>923</v>
       </c>
       <c r="T234" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="U234" t="s">
-        <v>922</v>
+        <v>924</v>
       </c>
     </row>
     <row r="235" spans="1:21">
       <c r="A235" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="B235" t="s">
-        <v>924</v>
+        <v>926</v>
       </c>
       <c r="C235" t="s">
-        <v>925</v>
+        <v>927</v>
       </c>
       <c r="D235">
         <v>2010</v>
@@ -16168,7 +16230,7 @@
         <v>40430</v>
       </c>
       <c r="S235" t="s">
-        <v>926</v>
+        <v>928</v>
       </c>
       <c r="T235" t="s">
         <v>26</v>
@@ -16176,13 +16238,13 @@
     </row>
     <row r="236" spans="1:21">
       <c r="A236" t="s">
-        <v>927</v>
+        <v>929</v>
       </c>
       <c r="B236" t="s">
-        <v>928</v>
+        <v>930</v>
       </c>
       <c r="C236" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="D236">
         <v>2011</v>
@@ -16200,7 +16262,7 @@
         <v>40782.520833333343</v>
       </c>
       <c r="I236" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="L236">
         <v>3.834384</v>
@@ -16220,7 +16282,7 @@
       <c r="Q236" s="2"/>
       <c r="R236" s="2"/>
       <c r="S236" t="s">
-        <v>929</v>
+        <v>931</v>
       </c>
       <c r="T236" t="s">
         <v>26</v>
@@ -16228,13 +16290,13 @@
     </row>
     <row r="237" spans="1:21">
       <c r="A237" t="s">
-        <v>930</v>
+        <v>932</v>
       </c>
       <c r="B237" t="s">
-        <v>931</v>
+        <v>933</v>
       </c>
       <c r="C237" t="s">
-        <v>932</v>
+        <v>934</v>
       </c>
       <c r="D237">
         <v>2012</v>
@@ -16252,7 +16314,7 @@
         <v>41150.291666666657</v>
       </c>
       <c r="I237" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="L237">
         <v>4.3433999999999999</v>
@@ -16276,7 +16338,7 @@
         <v>41153</v>
       </c>
       <c r="S237" t="s">
-        <v>933</v>
+        <v>935</v>
       </c>
       <c r="T237" t="s">
         <v>26</v>
@@ -16284,13 +16346,13 @@
     </row>
     <row r="238" spans="1:21">
       <c r="A238" t="s">
-        <v>934</v>
+        <v>936</v>
       </c>
       <c r="B238" t="s">
-        <v>935</v>
+        <v>937</v>
       </c>
       <c r="C238" t="s">
-        <v>936</v>
+        <v>938</v>
       </c>
       <c r="D238">
         <v>2012</v>
@@ -16308,7 +16370,7 @@
         <v>41211.979166666657</v>
       </c>
       <c r="I238" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="L238">
         <v>5.3279040000000002</v>
@@ -16331,13 +16393,13 @@
     </row>
     <row r="239" spans="1:21">
       <c r="A239" t="s">
-        <v>937</v>
+        <v>939</v>
       </c>
       <c r="B239" t="s">
-        <v>938</v>
+        <v>940</v>
       </c>
       <c r="C239" t="s">
-        <v>939</v>
+        <v>941</v>
       </c>
       <c r="D239">
         <v>2014</v>
@@ -16355,7 +16417,7 @@
         <v>41824.145833333343</v>
       </c>
       <c r="I239" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="L239">
         <v>2.1976079999999998</v>
@@ -16378,13 +16440,13 @@
     </row>
     <row r="240" spans="1:21">
       <c r="A240" t="s">
-        <v>940</v>
+        <v>942</v>
       </c>
       <c r="B240" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="C240" t="s">
-        <v>925</v>
+        <v>927</v>
       </c>
       <c r="D240">
         <v>2016</v>
@@ -16402,7 +16464,7 @@
         <v>42615.229166666657</v>
       </c>
       <c r="I240" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="L240">
         <v>3.148584</v>
@@ -16425,13 +16487,13 @@
     </row>
     <row r="241" spans="1:20">
       <c r="A241" t="s">
-        <v>942</v>
+        <v>944</v>
       </c>
       <c r="B241" t="s">
-        <v>943</v>
+        <v>945</v>
       </c>
       <c r="C241" t="s">
-        <v>944</v>
+        <v>946</v>
       </c>
       <c r="D241">
         <v>2016</v>
@@ -16478,13 +16540,13 @@
     </row>
     <row r="242" spans="1:20">
       <c r="A242" t="s">
-        <v>945</v>
+        <v>947</v>
       </c>
       <c r="B242" t="s">
-        <v>946</v>
+        <v>948</v>
       </c>
       <c r="C242" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="D242">
         <v>2017</v>
@@ -16531,13 +16593,13 @@
     </row>
     <row r="243" spans="1:20">
       <c r="A243" t="s">
-        <v>947</v>
+        <v>949</v>
       </c>
       <c r="B243" t="s">
-        <v>948</v>
+        <v>950</v>
       </c>
       <c r="C243" t="s">
-        <v>949</v>
+        <v>951</v>
       </c>
       <c r="D243">
         <v>2017</v>
@@ -16578,13 +16640,13 @@
     </row>
     <row r="244" spans="1:20">
       <c r="A244" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="B244" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
       <c r="C244" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="D244">
         <v>2017</v>
@@ -16602,7 +16664,7 @@
         <v>43016.229166666657</v>
       </c>
       <c r="I244" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="L244">
         <v>3.24003</v>

</xml_diff>